<commit_message>
release(v2.0): 2.0.0a4, Phase 2 trust gates and user manual (#1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Learnings Register" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Learning Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Learnings Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Recommendations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Learning Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="About" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3855,7 +3855,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a3</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5325,7 +5325,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a3</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6289,7 +6289,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a3</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6785,7 +6785,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a3</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6838,7 +6838,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Generated with ProbeMatrix Learnings Coach v2.0.0a3 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</t>
+          <t>Generated with ProbeMatrix Learnings Coach v2.0.0a4 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a3</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
release(v2.0): 2.0.0a5, Phase 3 shared spine and router (#1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
@@ -13,7 +13,11 @@
     <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="About" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Learnings Register'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Recommendations'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Learning Plan'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +36,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -59,10 +67,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -139,6 +150,75 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LearningsRegister" displayName="LearningsRegister" ref="A1:AB26" headerRowCount="1">
+  <autoFilter ref="A1:AB26"/>
+  <tableColumns count="28">
+    <tableColumn id="1" name="LR-ID"/>
+    <tableColumn id="2" name="ML-ID"/>
+    <tableColumn id="3" name="Title"/>
+    <tableColumn id="4" name="Learning cluster (entity)"/>
+    <tableColumn id="5" name="Tiers who must learn"/>
+    <tableColumn id="6" name="Lesson statement"/>
+    <tableColumn id="7" name="Context narrative"/>
+    <tableColumn id="8" name="Finding IDs"/>
+    <tableColumn id="9" name="Evidence IDs"/>
+    <tableColumn id="10" name="Evidence strength"/>
+    <tableColumn id="11" name="Confidence"/>
+    <tableColumn id="12" name="HFACS level / sub-category"/>
+    <tableColumn id="13" name="Causal role"/>
+    <tableColumn id="14" name="Barrier (prevention / mitigation)"/>
+    <tableColumn id="15" name="Hazard / energy"/>
+    <tableColumn id="16" name="Activity / phase"/>
+    <tableColumn id="17" name="Human-performance mode"/>
+    <tableColumn id="18" name="Organisational system"/>
+    <tableColumn id="19" name="Cross-incident / recurrence pattern"/>
+    <tableColumn id="20" name="Precursors and weak signals"/>
+    <tableColumn id="21" name="Counterpart in comparator report"/>
+    <tableColumn id="22" name="Reason class (if none)"/>
+    <tableColumn id="23" name="Credible worst case"/>
+    <tableColumn id="24" name="Transferability"/>
+    <tableColumn id="25" name="Priority"/>
+    <tableColumn id="26" name="Audiences"/>
+    <tableColumn id="27" name="Learning level / loop"/>
+    <tableColumn id="28" name="Formats"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Recommendations" displayName="Recommendations" ref="A1:F45" headerRowCount="1">
+  <autoFilter ref="A1:F45"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="LR-ID"/>
+    <tableColumn id="2" name="What should change"/>
+    <tableColumn id="3" name="HFACS level and barrier"/>
+    <tableColumn id="4" name="Evidence basis"/>
+    <tableColumn id="5" name="Hierarchy-of-controls tier"/>
+    <tableColumn id="6" name="Leading indicator"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="LearningPlan" displayName="LearningPlan" ref="A1:H26" headerRowCount="1">
+  <autoFilter ref="A1:H26"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="LR-ID"/>
+    <tableColumn id="2" name="Title"/>
+    <tableColumn id="3" name="Priority"/>
+    <tableColumn id="4" name="T1 Frontline"/>
+    <tableColumn id="5" name="T2 Supervisors"/>
+    <tableColumn id="6" name="T3 Function managers"/>
+    <tableColumn id="7" name="T4 Site leadership"/>
+    <tableColumn id="8" name="T5 Corporate / board"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -428,7 +508,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3852,15 +3932,27 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="Y2:Y26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"yes,partial,none,not compared"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3868,7 +3960,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3914,7 +4006,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>LR-01</t>
         </is>
@@ -3946,7 +4038,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>LR-01</t>
         </is>
@@ -3978,7 +4070,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>LR-01</t>
         </is>
@@ -4010,7 +4102,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>LR-02</t>
         </is>
@@ -4042,7 +4134,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>LR-02</t>
         </is>
@@ -4074,7 +4166,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>LR-03</t>
         </is>
@@ -4106,7 +4198,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>LR-03</t>
         </is>
@@ -4138,7 +4230,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>LR-04</t>
         </is>
@@ -4170,7 +4262,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>LR-04</t>
         </is>
@@ -4202,7 +4294,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>LR-05</t>
         </is>
@@ -4234,7 +4326,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>LR-05</t>
         </is>
@@ -4266,7 +4358,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>LR-06</t>
         </is>
@@ -4298,7 +4390,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>LR-06</t>
         </is>
@@ -4330,7 +4422,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>LR-07</t>
         </is>
@@ -4362,7 +4454,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>LR-07</t>
         </is>
@@ -4394,7 +4486,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>LR-07</t>
         </is>
@@ -4426,7 +4518,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>LR-08</t>
         </is>
@@ -4458,7 +4550,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>LR-08</t>
         </is>
@@ -4490,7 +4582,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>LR-09</t>
         </is>
@@ -4522,7 +4614,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>LR-09</t>
         </is>
@@ -4554,7 +4646,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>LR-10</t>
         </is>
@@ -4586,7 +4678,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>LR-10</t>
         </is>
@@ -4618,7 +4710,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>LR-11</t>
         </is>
@@ -4650,7 +4742,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>LR-11</t>
         </is>
@@ -4682,7 +4774,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>LR-12</t>
         </is>
@@ -4714,7 +4806,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>LR-12</t>
         </is>
@@ -4746,7 +4838,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>LR-13</t>
         </is>
@@ -4778,7 +4870,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>LR-13</t>
         </is>
@@ -4810,7 +4902,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>LR-14</t>
         </is>
@@ -4842,7 +4934,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>LR-15</t>
         </is>
@@ -4874,7 +4966,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>LR-15</t>
         </is>
@@ -4906,7 +4998,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>LR-16</t>
         </is>
@@ -4938,7 +5030,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>LR-16</t>
         </is>
@@ -4970,7 +5062,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>LR-17</t>
         </is>
@@ -5002,7 +5094,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>LR-17</t>
         </is>
@@ -5034,7 +5126,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>LR-18</t>
         </is>
@@ -5066,7 +5158,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>LR-19</t>
         </is>
@@ -5098,7 +5190,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>LR-20</t>
         </is>
@@ -5130,7 +5222,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>LR-21</t>
         </is>
@@ -5162,7 +5254,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>LR-22</t>
         </is>
@@ -5194,7 +5286,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>LR-23</t>
         </is>
@@ -5226,7 +5318,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>LR-23</t>
         </is>
@@ -5258,7 +5350,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>LR-24</t>
         </is>
@@ -5290,7 +5382,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>LR-25</t>
         </is>
@@ -5322,15 +5414,70 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"elimination,substitution,engineering,administrative,training,ppe"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Learnings Register'!A2"/>
+    <hyperlink ref="A3" location="'Learnings Register'!A2"/>
+    <hyperlink ref="A4" location="'Learnings Register'!A2"/>
+    <hyperlink ref="A5" location="'Learnings Register'!A3"/>
+    <hyperlink ref="A6" location="'Learnings Register'!A3"/>
+    <hyperlink ref="A7" location="'Learnings Register'!A4"/>
+    <hyperlink ref="A8" location="'Learnings Register'!A4"/>
+    <hyperlink ref="A9" location="'Learnings Register'!A5"/>
+    <hyperlink ref="A10" location="'Learnings Register'!A5"/>
+    <hyperlink ref="A11" location="'Learnings Register'!A6"/>
+    <hyperlink ref="A12" location="'Learnings Register'!A6"/>
+    <hyperlink ref="A13" location="'Learnings Register'!A7"/>
+    <hyperlink ref="A14" location="'Learnings Register'!A7"/>
+    <hyperlink ref="A15" location="'Learnings Register'!A8"/>
+    <hyperlink ref="A16" location="'Learnings Register'!A8"/>
+    <hyperlink ref="A17" location="'Learnings Register'!A8"/>
+    <hyperlink ref="A18" location="'Learnings Register'!A9"/>
+    <hyperlink ref="A19" location="'Learnings Register'!A9"/>
+    <hyperlink ref="A20" location="'Learnings Register'!A10"/>
+    <hyperlink ref="A21" location="'Learnings Register'!A10"/>
+    <hyperlink ref="A22" location="'Learnings Register'!A11"/>
+    <hyperlink ref="A23" location="'Learnings Register'!A11"/>
+    <hyperlink ref="A24" location="'Learnings Register'!A12"/>
+    <hyperlink ref="A25" location="'Learnings Register'!A12"/>
+    <hyperlink ref="A26" location="'Learnings Register'!A13"/>
+    <hyperlink ref="A27" location="'Learnings Register'!A13"/>
+    <hyperlink ref="A28" location="'Learnings Register'!A14"/>
+    <hyperlink ref="A29" location="'Learnings Register'!A14"/>
+    <hyperlink ref="A30" location="'Learnings Register'!A15"/>
+    <hyperlink ref="A31" location="'Learnings Register'!A16"/>
+    <hyperlink ref="A32" location="'Learnings Register'!A16"/>
+    <hyperlink ref="A33" location="'Learnings Register'!A17"/>
+    <hyperlink ref="A34" location="'Learnings Register'!A17"/>
+    <hyperlink ref="A35" location="'Learnings Register'!A18"/>
+    <hyperlink ref="A36" location="'Learnings Register'!A18"/>
+    <hyperlink ref="A37" location="'Learnings Register'!A19"/>
+    <hyperlink ref="A38" location="'Learnings Register'!A20"/>
+    <hyperlink ref="A39" location="'Learnings Register'!A21"/>
+    <hyperlink ref="A40" location="'Learnings Register'!A22"/>
+    <hyperlink ref="A41" location="'Learnings Register'!A23"/>
+    <hyperlink ref="A42" location="'Learnings Register'!A24"/>
+    <hyperlink ref="A43" location="'Learnings Register'!A24"/>
+    <hyperlink ref="A44" location="'Learnings Register'!A25"/>
+    <hyperlink ref="A45" location="'Learnings Register'!A26"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -5338,7 +5485,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6287,14 +6434,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -6302,7 +6453,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6783,9 +6934,10 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6798,12 +6950,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="200" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -6838,7 +6990,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Generated with ProbeMatrix Learnings Coach v2.0.0a4 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</t>
+          <t>Generated with ProbeMatrix Learnings Coach v2.0.0a5 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</t>
         </is>
       </c>
     </row>
@@ -6916,9 +7068,10 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a4</oddFooter>
+    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
release(v2.0): 2.0.0a6, Phase 4 outputs (#1)
Version 2.0.0a6 (2.0.0-alpha.6) via tools/release.py; goldens and the
Hazira samples re-rendered at 2026-10-22 (version and date stamps only);
CHANGELOG records the measured blind routing, the png --no-sandbox retry,
brand masking in shared copies and the interview-plan cap of 31.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
@@ -3944,7 +3944,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5469,7 +5469,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6437,7 +6437,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6937,7 +6937,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6990,7 +6990,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Generated with ProbeMatrix Learnings Coach v2.0.0a5 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</t>
+          <t>Generated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CProbeMatrix Learnings Coach v2.0.0a5</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
fix(engine): refresh Hazira register renders, pin check-register, reword manual (#1)
Regenerate learnings-register.xlsx and organisation-learning-map.html from the
updated register JSON; record 205 as the distinct single-source count; assert
the sample register gives 0 problems.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
@@ -863,7 +863,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>inferred</t>
+          <t>corroborated</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(samples): Hazira golden packs for the Phase 6 skills (#1)
Render the seven Phase 6 goldens (html, md) and the showcases: the
safety-alert poster and pptx, the safety-moment-deck pptx, the AcciMap
svg, the CIHH return template and the blank learning-team notes. The
register workbook and dashboard are re-rendered from the urgency
register. RENDER_PENDING is empty again; group F pins check-pack
--strict and check-language for the seven packs, the register's 0
problems, the blank organisation columns and the fresh register files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011J2b33mikuz2J1RKTx4krR
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/learnings-register.xlsx
@@ -153,9 +153,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LearningsRegister" displayName="LearningsRegister" ref="A1:AB26" headerRowCount="1">
-  <autoFilter ref="A1:AB26"/>
-  <tableColumns count="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LearningsRegister" displayName="LearningsRegister" ref="A1:AC26" headerRowCount="1">
+  <autoFilter ref="A1:AC26"/>
+  <tableColumns count="29">
     <tableColumn id="1" name="LR-ID"/>
     <tableColumn id="2" name="ML-ID"/>
     <tableColumn id="3" name="Title"/>
@@ -184,6 +184,7 @@
     <tableColumn id="26" name="Audiences"/>
     <tableColumn id="27" name="Learning level / loop"/>
     <tableColumn id="28" name="Formats"/>
+    <tableColumn id="29" name="Urgency"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -510,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB26"/>
+  <dimension ref="A1:AC26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -541,6 +542,7 @@
     <col width="18" customWidth="1" min="26" max="26"/>
     <col width="32" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -684,6 +686,11 @@
           <t>Formats</t>
         </is>
       </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Urgency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -818,6 +825,11 @@
           <t>Brief; Card; toolbox talk</t>
         </is>
       </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -952,6 +964,11 @@
           <t>Card; toolbox talk; Brief</t>
         </is>
       </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1082,6 +1099,11 @@
           <t>Card; Brief</t>
         </is>
       </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1216,6 +1238,11 @@
           <t>Card</t>
         </is>
       </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1350,6 +1377,11 @@
           <t>Brief; Card</t>
         </is>
       </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1484,6 +1516,11 @@
           <t>Brief; toolbox talk</t>
         </is>
       </c>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1612,6 +1649,11 @@
       <c r="AB8" s="2" t="inlineStr">
         <is>
           <t>Brief; Card; toolbox talk; module</t>
+        </is>
+      </c>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
         </is>
       </c>
     </row>
@@ -1740,6 +1782,11 @@
           <t>Card; toolbox talk; module</t>
         </is>
       </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1868,6 +1915,11 @@
       <c r="AB10" s="2" t="inlineStr">
         <is>
           <t>Brief</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
         </is>
       </c>
     </row>
@@ -1996,6 +2048,11 @@
           <t>Brief</t>
         </is>
       </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2126,6 +2183,11 @@
           <t>Card; toolbox talk</t>
         </is>
       </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2256,6 +2318,11 @@
           <t>Brief; module</t>
         </is>
       </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2384,6 +2451,11 @@
       <c r="AB14" s="2" t="inlineStr">
         <is>
           <t>Card; toolbox talk</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
         </is>
       </c>
     </row>
@@ -2512,6 +2584,11 @@
           <t>Brief</t>
         </is>
       </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2638,6 +2715,11 @@
           <t>Card</t>
         </is>
       </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2768,6 +2850,11 @@
           <t>Card</t>
         </is>
       </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2902,6 +2989,11 @@
           <t>Brief</t>
         </is>
       </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3030,6 +3122,11 @@
       <c r="AB19" s="2" t="inlineStr">
         <is>
           <t>Brief</t>
+        </is>
+      </c>
+      <c r="AC19" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
         </is>
       </c>
     </row>
@@ -3158,6 +3255,11 @@
           <t>Brief</t>
         </is>
       </c>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3292,6 +3394,11 @@
           <t>Brief</t>
         </is>
       </c>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3422,6 +3529,11 @@
           <t>Brief</t>
         </is>
       </c>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>information</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3550,6 +3662,11 @@
       <c r="AB23" s="2" t="inlineStr">
         <is>
           <t>Card; toolbox talk</t>
+        </is>
+      </c>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
         </is>
       </c>
     </row>
@@ -3678,6 +3795,11 @@
           <t>Card; Brief</t>
         </is>
       </c>
+      <c r="AC24" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3804,6 +3926,11 @@
           <t>Card</t>
         </is>
       </c>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>information</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3928,6 +4055,11 @@
       <c r="AB26" s="2" t="inlineStr">
         <is>
           <t>Brief</t>
+        </is>
+      </c>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>notice</t>
         </is>
       </c>
     </row>

</xml_diff>